<commit_message>
Convert performance-ratios template to student exercise
Blank the 29 ratio formulas in column C (rows 43-76) so students compute
them using the named-range formulas shown in column D. Keep upstream
plumbing (start-of-year lookups, derived current-year inputs, averages)
prefilled to avoid blocking on data wiring.

Add a Self-checks block on the Notes sheet covering Du Pont ROA (exact
match to direct ROA) and Du Pont ROE (won't match - framed as a Stage 4
memo prompt explaining the time-mismatch). Add an inline check cell at
Ratios!F75 that confirms Du Pont ROA matches direct ROA once filled in.

Update Stage 3 task description on Notes to reflect that students now
compute ratios, not just enter assumptions.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/spreadsheets/performance-ratios-template.xlsx
+++ b/docs/templates/spreadsheets/performance-ratios-template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="600" firstSheet="1" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
@@ -23,8 +23,8 @@
     <definedName name="BAL_accumulated_depreciation_prior">'Balance Sheet'!$D$15</definedName>
     <definedName name="BAL_assets_current_curr">'Balance Sheet'!$C$11</definedName>
     <definedName name="BAL_assets_current_prior">'Balance Sheet'!$D$11</definedName>
-    <definedName name="BAL_assets_total_curr">'Balance Sheet'!$C$22</definedName>
-    <definedName name="BAL_assets_total_prior">'Balance Sheet'!$D$22</definedName>
+    <definedName name="BAL_assets_total_curr">'Balance Sheet'!$C$23</definedName>
+    <definedName name="BAL_assets_total_prior">'Balance Sheet'!$D$23</definedName>
     <definedName name="BAL_cash_marketable_securities_curr">'Balance Sheet'!$C$7</definedName>
     <definedName name="BAL_cash_marketable_securities_prior">'Balance Sheet'!$D$7</definedName>
     <definedName name="BAL_common_stock_curr">'Balance Sheet'!$G$18</definedName>
@@ -118,7 +118,7 @@
     <numFmt numFmtId="170" formatCode="0.0&quot; days&quot;"/>
     <numFmt numFmtId="171" formatCode="0.000"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -225,6 +225,11 @@
       <color rgb="FF024731"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Open Sans"/>
+      <color rgb="FF024731"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -297,7 +302,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -374,21 +379,17 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+    <xf numFmtId="49" fontId="18" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -769,21 +770,21 @@
       <c r="C2" s="1" t="n"/>
     </row>
     <row r="4">
-      <c r="B4" s="49" t="inlineStr">
+      <c r="B4" s="50" t="inlineStr">
         <is>
           <t>UNIVERSITY OF HAWAIʻI AT MĀNOA · SHIDLER COLLEGE OF BUSINESS</t>
         </is>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1" s="45">
-      <c r="B5" s="47" t="inlineStr">
+      <c r="B5" s="48" t="inlineStr">
         <is>
           <t>BUS-629 International Corporate Finance · Vietnam EMBA</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" s="45">
-      <c r="B6" s="44" t="inlineStr">
+      <c r="B6" s="46" t="inlineStr">
         <is>
           <t>Performance Ratios — Excel Template</t>
         </is>
@@ -794,7 +795,7 @@
       <c r="C7" s="2" t="n"/>
     </row>
     <row r="9" ht="19.5" customHeight="1" s="45">
-      <c r="B9" s="46" t="inlineStr">
+      <c r="B9" s="47" t="inlineStr">
         <is>
           <t>How to Use This Template</t>
         </is>
@@ -873,7 +874,7 @@
       </c>
     </row>
     <row r="17" ht="19.5" customHeight="1" s="45">
-      <c r="B17" s="46" t="inlineStr">
+      <c r="B17" s="47" t="inlineStr">
         <is>
           <t>Color Key</t>
         </is>
@@ -940,7 +941,7 @@
       </c>
     </row>
     <row r="24" ht="19.5" customHeight="1" s="45">
-      <c r="B24" s="46" t="inlineStr">
+      <c r="B24" s="47" t="inlineStr">
         <is>
           <t>Named-Range Convention</t>
         </is>
@@ -1055,7 +1056,7 @@
       </c>
     </row>
     <row r="36" ht="19.5" customHeight="1" s="45">
-      <c r="B36" s="46" t="inlineStr">
+      <c r="B36" s="47" t="inlineStr">
         <is>
           <t>Companion Specification</t>
         </is>
@@ -1086,7 +1087,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="48" t="inlineStr">
+      <c r="B41" s="49" t="inlineStr">
         <is>
           <t>Prepared per UH Mānoa brand standards (docs/_branding/design.json). Primary green #024731 · Open Sans typography · ADA-compliant contrast.</t>
         </is>
@@ -1395,22 +1396,21 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="45">
-      <c r="B22" s="5" t="inlineStr">
+    <row r="22" ht="16.5" customHeight="1" s="45"/>
+    <row r="23" ht="16.5" customHeight="1" s="45">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Total Assets</t>
         </is>
       </c>
-      <c r="C22" s="22">
+      <c r="C23" s="22">
         <f>C11+C16+C19+C20</f>
         <v/>
       </c>
-      <c r="D22" s="22">
+      <c r="D23" s="22">
         <f>D11+D16+D19+D20</f>
         <v/>
       </c>
-    </row>
-    <row r="23" ht="16.5" customHeight="1" s="45">
       <c r="F23" s="5" t="inlineStr">
         <is>
           <t>Total Liabilities + Equity</t>
@@ -1483,7 +1483,7 @@
         </is>
       </c>
       <c r="C6" s="19" t="n"/>
-      <c r="D6" s="51" t="n">
+      <c r="D6" s="24" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
         </is>
       </c>
       <c r="C7" s="19" t="n"/>
-      <c r="D7" s="52">
+      <c r="D7" s="25">
         <f>IFERROR(C7/$C$6,"")</f>
         <v/>
       </c>
@@ -1506,7 +1506,7 @@
         </is>
       </c>
       <c r="C8" s="19" t="n"/>
-      <c r="D8" s="52">
+      <c r="D8" s="25">
         <f>IFERROR(C8/$C$6,"")</f>
         <v/>
       </c>
@@ -1518,7 +1518,7 @@
         </is>
       </c>
       <c r="C9" s="19" t="n"/>
-      <c r="D9" s="52">
+      <c r="D9" s="25">
         <f>IFERROR(C9/$C$6,"")</f>
         <v/>
       </c>
@@ -1533,7 +1533,7 @@
         <f>C6-C7-C8-C9</f>
         <v/>
       </c>
-      <c r="D10" s="52">
+      <c r="D10" s="25">
         <f>IFERROR(C10/$C$6,"")</f>
         <v/>
       </c>
@@ -1545,7 +1545,7 @@
         </is>
       </c>
       <c r="C11" s="19" t="n"/>
-      <c r="D11" s="52">
+      <c r="D11" s="25">
         <f>IFERROR(C11/$C$6,"")</f>
         <v/>
       </c>
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="C12" s="19" t="n"/>
-      <c r="D12" s="52">
+      <c r="D12" s="25">
         <f>IFERROR(C12/$C$6,"")</f>
         <v/>
       </c>
@@ -1572,7 +1572,7 @@
         <f>C10+C11-C12</f>
         <v/>
       </c>
-      <c r="D13" s="52">
+      <c r="D13" s="25">
         <f>IFERROR(C13/$C$6,"")</f>
         <v/>
       </c>
@@ -1584,7 +1584,7 @@
         </is>
       </c>
       <c r="C14" s="19" t="n"/>
-      <c r="D14" s="52">
+      <c r="D14" s="25">
         <f>IFERROR(C14/$C$6,"")</f>
         <v/>
       </c>
@@ -1599,7 +1599,7 @@
         <f>C13-C14</f>
         <v/>
       </c>
-      <c r="D15" s="53">
+      <c r="D15" s="26">
         <f>IFERROR(C15/$C$6,"")</f>
         <v/>
       </c>
@@ -1618,7 +1618,7 @@
         </is>
       </c>
       <c r="C18" s="19" t="n"/>
-      <c r="D18" s="52">
+      <c r="D18" s="25">
         <f>IFERROR(C18/$C$6,"")</f>
         <v/>
       </c>
@@ -1633,7 +1633,7 @@
         <f>C15-C18</f>
         <v/>
       </c>
-      <c r="D19" s="52">
+      <c r="D19" s="25">
         <f>IFERROR(C19/$C$6,"")</f>
         <v/>
       </c>
@@ -1970,7 +1970,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E76"/>
+  <dimension ref="B2:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="2" customWidth="1" style="45" min="1" max="1"/>
@@ -1978,6 +1978,7 @@
     <col width="16" customWidth="1" style="45" min="3" max="3"/>
     <col width="62" customWidth="1" style="45" min="4" max="4"/>
     <col width="36" customWidth="1" style="45" min="5" max="5"/>
+    <col width="28" customWidth="1" style="45" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="2" ht="23" customHeight="1" s="45">
@@ -2087,7 +2088,7 @@
           <t>Cost of capital</t>
         </is>
       </c>
-      <c r="C10" s="54" t="n">
+      <c r="C10" s="34" t="n">
         <v>0.09</v>
       </c>
       <c r="D10" s="30" t="n"/>
@@ -2103,7 +2104,7 @@
           <t>Tax rate</t>
         </is>
       </c>
-      <c r="C11" s="54" t="n">
+      <c r="C11" s="34" t="n">
         <v>0.21</v>
       </c>
       <c r="D11" s="30" t="n"/>
@@ -2135,7 +2136,7 @@
       </c>
     </row>
     <row r="14" ht="16.5" customHeight="1" s="45">
-      <c r="B14" s="50" t="inlineStr">
+      <c r="B14" s="44" t="inlineStr">
         <is>
           <t>── Start of Year (Prior-Year Balance Sheet) ──</t>
         </is>
@@ -2247,7 +2248,7 @@
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1" s="45">
-      <c r="B21" s="50" t="inlineStr">
+      <c r="B21" s="44" t="inlineStr">
         <is>
           <t>── Current Year (Derived) ──</t>
         </is>
@@ -2506,7 +2507,7 @@
       </c>
     </row>
     <row r="35" ht="16.5" customHeight="1" s="45">
-      <c r="B35" s="50" t="inlineStr">
+      <c r="B35" s="44" t="inlineStr">
         <is>
           <t>── Mixed Year (Averages) ──</t>
         </is>
@@ -2594,6 +2595,11 @@
       <c r="E41" s="23" t="inlineStr">
         <is>
           <t>Named Range</t>
+        </is>
+      </c>
+      <c r="F41" s="23" t="inlineStr">
+        <is>
+          <t>Check</t>
         </is>
       </c>
     </row>
@@ -2613,10 +2619,7 @@
           <t>Market value added (MVA)</t>
         </is>
       </c>
-      <c r="C43" s="38">
-        <f>market_capitalization-currentYear_equity</f>
-        <v/>
-      </c>
+      <c r="C43" s="38" t="n"/>
       <c r="D43" s="30" t="inlineStr">
         <is>
           <t>market_capitalization − currentYear_equity</t>
@@ -2630,10 +2633,7 @@
           <t>Market-to-book ratio</t>
         </is>
       </c>
-      <c r="C44" s="39">
-        <f>IFERROR(market_capitalization/currentYear_equity,"")</f>
-        <v/>
-      </c>
+      <c r="C44" s="39" t="n"/>
       <c r="D44" s="30" t="inlineStr">
         <is>
           <t>market_capitalization / currentYear_equity</t>
@@ -2647,10 +2647,7 @@
           <t>Economic value added (EVA)</t>
         </is>
       </c>
-      <c r="C45" s="38">
-        <f>currentYear_after_tax_operating_income-(cost_capital*startYear_total_capitalization)</f>
-        <v/>
-      </c>
+      <c r="C45" s="38" t="n"/>
       <c r="D45" s="30" t="inlineStr">
         <is>
           <t>currentYear_after_tax_operating_income − (cost_capital × startYear_total_capitalization)</t>
@@ -2674,10 +2671,7 @@
           <t>Return on assets (ROA)</t>
         </is>
       </c>
-      <c r="C47" s="55">
-        <f>IFERROR(currentYear_after_tax_operating_income/startYear_total_assets,"")</f>
-        <v/>
-      </c>
+      <c r="C47" s="40" t="n"/>
       <c r="D47" s="30" t="inlineStr">
         <is>
           <t>currentYear_after_tax_operating_income / startYear_total_assets</t>
@@ -2691,10 +2685,7 @@
           <t>Return on capital (ROC)</t>
         </is>
       </c>
-      <c r="C48" s="55">
-        <f>IFERROR(currentYear_after_tax_operating_income/startYear_total_capitalization,"")</f>
-        <v/>
-      </c>
+      <c r="C48" s="40" t="n"/>
       <c r="D48" s="30" t="inlineStr">
         <is>
           <t>currentYear_after_tax_operating_income / startYear_total_capitalization</t>
@@ -2708,10 +2699,7 @@
           <t>Return on equity (ROE)</t>
         </is>
       </c>
-      <c r="C49" s="55">
-        <f>IFERROR(INC_net/startYear_equity,"")</f>
-        <v/>
-      </c>
+      <c r="C49" s="40" t="n"/>
       <c r="D49" s="30" t="inlineStr">
         <is>
           <t>INC_net / startYear_equity</t>
@@ -2725,10 +2713,7 @@
           <t>Return on assets (ROA) [avg]</t>
         </is>
       </c>
-      <c r="C50" s="55">
-        <f>IFERROR(currentYear_after_tax_operating_income/avg_total_assets,"")</f>
-        <v/>
-      </c>
+      <c r="C50" s="40" t="n"/>
       <c r="D50" s="30" t="inlineStr">
         <is>
           <t>currentYear_after_tax_operating_income / avg_total_assets</t>
@@ -2742,10 +2727,7 @@
           <t>Return on capital (ROC) [avg]</t>
         </is>
       </c>
-      <c r="C51" s="55">
-        <f>IFERROR(currentYear_after_tax_operating_income/avg_total_capitalization,"")</f>
-        <v/>
-      </c>
+      <c r="C51" s="40" t="n"/>
       <c r="D51" s="30" t="inlineStr">
         <is>
           <t>currentYear_after_tax_operating_income / avg_total_capitalization</t>
@@ -2759,10 +2741,7 @@
           <t>Return on equity (ROE) [avg]</t>
         </is>
       </c>
-      <c r="C52" s="55">
-        <f>IFERROR(INC_net/avg_equity,"")</f>
-        <v/>
-      </c>
+      <c r="C52" s="40" t="n"/>
       <c r="D52" s="30" t="inlineStr">
         <is>
           <t>INC_net / avg_equity</t>
@@ -2786,10 +2765,7 @@
           <t>Asset turnover</t>
         </is>
       </c>
-      <c r="C54" s="39">
-        <f>IFERROR(INC_sales/startYear_total_assets,"")</f>
-        <v/>
-      </c>
+      <c r="C54" s="39" t="n"/>
       <c r="D54" s="30" t="inlineStr">
         <is>
           <t>INC_sales / startYear_total_assets</t>
@@ -2807,10 +2783,7 @@
           <t>Receivables turnover</t>
         </is>
       </c>
-      <c r="C55" s="39">
-        <f>IFERROR(INC_sales/startYear_receivables,"")</f>
-        <v/>
-      </c>
+      <c r="C55" s="39" t="n"/>
       <c r="D55" s="30" t="inlineStr">
         <is>
           <t>INC_sales / startYear_receivables</t>
@@ -2824,10 +2797,7 @@
           <t>Average collection period (days)</t>
         </is>
       </c>
-      <c r="C56" s="41">
-        <f>IFERROR(startYear_receivables/currentYear_daily_sales_average,"")</f>
-        <v/>
-      </c>
+      <c r="C56" s="41" t="n"/>
       <c r="D56" s="30" t="inlineStr">
         <is>
           <t>startYear_receivables / currentYear_daily_sales_average</t>
@@ -2841,10 +2811,7 @@
           <t>Inventory turnover</t>
         </is>
       </c>
-      <c r="C57" s="39">
-        <f>IFERROR(INC_cost_goods_sold/startYear_inventory,"")</f>
-        <v/>
-      </c>
+      <c r="C57" s="39" t="n"/>
       <c r="D57" s="30" t="inlineStr">
         <is>
           <t>INC_cost_goods_sold / startYear_inventory</t>
@@ -2858,10 +2825,7 @@
           <t>Days in inventory</t>
         </is>
       </c>
-      <c r="C58" s="41">
-        <f>IFERROR(startYear_inventory/currentYear_cost_goods_sold_daily,"")</f>
-        <v/>
-      </c>
+      <c r="C58" s="41" t="n"/>
       <c r="D58" s="30" t="inlineStr">
         <is>
           <t>startYear_inventory / currentYear_cost_goods_sold_daily</t>
@@ -2875,10 +2839,7 @@
           <t>Profit margin</t>
         </is>
       </c>
-      <c r="C59" s="55">
-        <f>IFERROR(INC_net/INC_sales,"")</f>
-        <v/>
-      </c>
+      <c r="C59" s="40" t="n"/>
       <c r="D59" s="30" t="inlineStr">
         <is>
           <t>INC_net / INC_sales</t>
@@ -2892,10 +2853,7 @@
           <t>Operating profit margin</t>
         </is>
       </c>
-      <c r="C60" s="55">
-        <f>IFERROR(currentYear_after_tax_operating_income/INC_sales,"")</f>
-        <v/>
-      </c>
+      <c r="C60" s="40" t="n"/>
       <c r="D60" s="30" t="inlineStr">
         <is>
           <t>currentYear_after_tax_operating_income / INC_sales</t>
@@ -2923,10 +2881,7 @@
           <t>Long-term debt ratio</t>
         </is>
       </c>
-      <c r="C62" s="55">
-        <f>IFERROR(currentYear_debt_long_term/(currentYear_debt_long_term+currentYear_equity),"")</f>
-        <v/>
-      </c>
+      <c r="C62" s="40" t="n"/>
       <c r="D62" s="30" t="inlineStr">
         <is>
           <t>currentYear_debt_long_term / (currentYear_debt_long_term + currentYear_equity)</t>
@@ -2940,10 +2895,7 @@
           <t>Long-term debt-equity ratio</t>
         </is>
       </c>
-      <c r="C63" s="39">
-        <f>IFERROR(currentYear_debt_long_term/currentYear_equity,"")</f>
-        <v/>
-      </c>
+      <c r="C63" s="39" t="n"/>
       <c r="D63" s="30" t="inlineStr">
         <is>
           <t>currentYear_debt_long_term / currentYear_equity</t>
@@ -2957,10 +2909,7 @@
           <t>Total debt ratio</t>
         </is>
       </c>
-      <c r="C64" s="55">
-        <f>IFERROR(currentYear_liabilities_total/currentYear_assets_total,"")</f>
-        <v/>
-      </c>
+      <c r="C64" s="40" t="n"/>
       <c r="D64" s="30" t="inlineStr">
         <is>
           <t>currentYear_liabilities_total / currentYear_assets_total</t>
@@ -2974,10 +2923,7 @@
           <t>Times interest earned</t>
         </is>
       </c>
-      <c r="C65" s="39">
-        <f>IFERROR(INC_ebit/INC_interest_expense,"")</f>
-        <v/>
-      </c>
+      <c r="C65" s="39" t="n"/>
       <c r="D65" s="30" t="inlineStr">
         <is>
           <t>INC_ebit / INC_interest_expense</t>
@@ -2991,10 +2937,7 @@
           <t>Cash coverage ratio</t>
         </is>
       </c>
-      <c r="C66" s="39">
-        <f>IFERROR((INC_ebit+INC_depreciation)/INC_interest_expense,"")</f>
-        <v/>
-      </c>
+      <c r="C66" s="39" t="n"/>
       <c r="D66" s="30" t="inlineStr">
         <is>
           <t>(INC_ebit + INC_depreciation) / INC_interest_expense</t>
@@ -3008,10 +2951,7 @@
           <t>Debt burden</t>
         </is>
       </c>
-      <c r="C67" s="42">
-        <f>IFERROR(INC_net/currentYear_after_tax_operating_income,"")</f>
-        <v/>
-      </c>
+      <c r="C67" s="42" t="n"/>
       <c r="D67" s="30" t="inlineStr">
         <is>
           <t>INC_net / currentYear_after_tax_operating_income</t>
@@ -3029,10 +2969,7 @@
           <t>Leverage ratio</t>
         </is>
       </c>
-      <c r="C68" s="39">
-        <f>IFERROR(currentYear_assets_total/currentYear_equity,"")</f>
-        <v/>
-      </c>
+      <c r="C68" s="39" t="n"/>
       <c r="D68" s="30" t="inlineStr">
         <is>
           <t>currentYear_assets_total / currentYear_equity</t>
@@ -3060,10 +2997,7 @@
           <t>Net working capital to assets</t>
         </is>
       </c>
-      <c r="C70" s="55">
-        <f>IFERROR(currentYear_working_capital_net/currentYear_assets_total,"")</f>
-        <v/>
-      </c>
+      <c r="C70" s="40" t="n"/>
       <c r="D70" s="30" t="inlineStr">
         <is>
           <t>currentYear_working_capital_net / currentYear_assets_total</t>
@@ -3077,10 +3011,7 @@
           <t>Current ratio</t>
         </is>
       </c>
-      <c r="C71" s="39">
-        <f>IFERROR(currentYear_assets_current/currentYear_liabilities_current,"")</f>
-        <v/>
-      </c>
+      <c r="C71" s="39" t="n"/>
       <c r="D71" s="30" t="inlineStr">
         <is>
           <t>currentYear_assets_current / currentYear_liabilities_current</t>
@@ -3094,10 +3025,7 @@
           <t>Quick ratio</t>
         </is>
       </c>
-      <c r="C72" s="39">
-        <f>IFERROR((currentYear_cash_marketable_securities+BAL_receivables_curr)/currentYear_liabilities_current,"")</f>
-        <v/>
-      </c>
+      <c r="C72" s="39" t="n"/>
       <c r="D72" s="30" t="inlineStr">
         <is>
           <t>(currentYear_cash_marketable_securities + BAL_receivables_curr) / currentYear_liabilities_current</t>
@@ -3111,10 +3039,7 @@
           <t>Cash ratio</t>
         </is>
       </c>
-      <c r="C73" s="39">
-        <f>IFERROR(currentYear_cash_marketable_securities/currentYear_liabilities_current,"")</f>
-        <v/>
-      </c>
+      <c r="C73" s="39" t="n"/>
       <c r="D73" s="30" t="inlineStr">
         <is>
           <t>currentYear_cash_marketable_securities / currentYear_liabilities_current</t>
@@ -3138,16 +3063,17 @@
           <t>Return on assets (Du Pont)</t>
         </is>
       </c>
-      <c r="C75" s="55">
-        <f>IFERROR(RATIO_asset_turnover*RATIO_operating_profit_margin,"")</f>
-        <v/>
-      </c>
+      <c r="C75" s="40" t="n"/>
       <c r="D75" s="30" t="inlineStr">
         <is>
           <t>RATIO_asset_turnover × RATIO_operating_profit_margin</t>
         </is>
       </c>
       <c r="E75" s="30" t="n"/>
+      <c r="F75" s="51">
+        <f>IF(OR(C75="",C47=""),"",IF(ROUND(C75,6)=ROUND(C47,6),"✓ matches direct ROA","✗ differs by "&amp;TEXT(ABS(C75-C47),"0.00%")))</f>
+        <v/>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="45">
       <c r="B76" s="12" t="inlineStr">
@@ -3155,10 +3081,7 @@
           <t>Return on equity (Du Pont)</t>
         </is>
       </c>
-      <c r="C76" s="55">
-        <f>IFERROR(RATIO_leverage*RATIO_asset_turnover*RATIO_operating_profit_margin*RATIO_debt_burden,"")</f>
-        <v/>
-      </c>
+      <c r="C76" s="40" t="n"/>
       <c r="D76" s="30" t="inlineStr">
         <is>
           <t>RATIO_leverage × RATIO_asset_turnover × RATIO_operating_profit_margin × RATIO_debt_burden</t>
@@ -3182,10 +3105,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:C20"/>
+  <dimension ref="B2:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="2" customWidth="1" style="45" min="1" max="1"/>
+    <col width="3.90625" customWidth="1" style="45" min="1" max="1"/>
     <col width="28" customWidth="1" style="45" min="2" max="2"/>
     <col width="70" customWidth="1" style="45" min="3" max="3"/>
   </cols>
@@ -3330,16 +3253,11 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="B16" s="43" t="inlineStr">
         <is>
           <t>BUS-629 Project Use</t>
         </is>
       </c>
-      <c r="B16" s="43" t="inlineStr">
-        <is>
-          <t>BUS-314 Project Use</t>
-        </is>
-      </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Template for the Accounting &amp; Performance Ratios project</t>
@@ -3347,11 +3265,6 @@
       </c>
     </row>
     <row r="17" ht="29" customHeight="1" s="45">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Stage 1 Task</t>
-        </is>
-      </c>
       <c r="B17" s="43" t="inlineStr">
         <is>
           <t>Stage 2 Task</t>
@@ -3363,46 +3276,31 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="18" ht="29" customHeight="1" s="45">
+      <c r="B18" s="43" t="inlineStr">
         <is>
           <t>Stage 3 Task</t>
         </is>
       </c>
-      <c r="B18" s="43" t="inlineStr">
-        <is>
-          <t>Stage 3 Task</t>
-        </is>
-      </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Populate Balance Sheet, Income Statement, Cash Flow, and Ratios-tab assumptions for your selected company.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+          <t>Populate Balance Sheet, Income Statement, and Cash Flow with your selected company’s figures; enter the four assumptions on the Ratios tab; then compute all ratios in column C using the named-range formulas shown in column D.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="29" customHeight="1" s="45">
+      <c r="B19" s="43" t="inlineStr">
         <is>
           <t>Stage 4 Task</t>
         </is>
       </c>
-      <c r="B19" s="43" t="inlineStr">
-        <is>
-          <t>Stage 4 Task</t>
-        </is>
-      </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Use an LLM to draft a technical specification (spec-template.md) covering this model and the analysis it should produce.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Stage 5 Task</t>
-        </is>
-      </c>
+    <row r="20" ht="29" customHeight="1" s="45">
       <c r="B20" s="43" t="inlineStr">
         <is>
           <t>AI Usage</t>
@@ -3411,6 +3309,37 @@
       <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Execute spec with LLM; evaluate output; ship final analysis as part of polished portfolio repo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="43" t="inlineStr">
+        <is>
+          <t>Self-checks</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1" s="45">
+      <c r="B23" s="43" t="inlineStr">
+        <is>
+          <t>Du Pont ROA</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Du Pont ROA (Ratios!C75) is mathematically identical to direct ROA (Ratios!C47). The inline check on Ratios!F75 confirms the match — investigate any discrepancy before submitting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="45" customHeight="1" s="45">
+      <c r="B24" s="43" t="inlineStr">
+        <is>
+          <t>Du Pont ROE</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Du Pont ROE (Ratios!C76) will not exactly equal direct ROE (Ratios!C49) in this model: the leverage component uses current-year balances while asset turnover uses prior-year assets. Explain this time-mismatch in your Stage 4 memo.</t>
         </is>
       </c>
     </row>

</xml_diff>